<commit_message>
feat(universitetlar): kasbiy ta'lim Excel'i va bakalavr / magistr / kasbiy ta'lim filtri
- Excel shablonida yangi daraja: kasbiy (전문대학, 전문학사). Katalog
  sarlavhasiga "Excel kasbiy" tugmasi, universitet paneliga
  "Kasbiy ta'lim" yorlig'i qo'shildi. university_guidelines.daraja
  cheklovi kengaytirildi (migratsiya).
- Daraja filtri: Barcha darajalar / Bakalavr / Magistr / Kasbiy ta'lim,
  yonida natija soni bilan. Universitet qaysi darajada o'qitishi
  yuklangan Excel'dan va oliygoh turidan aniqlanadi: kollej - kasbiy
  ta'lim, 대학원대학교 - faqat magistr, qolganlari - bakalavr va magistr.
  Daraja tanlansa, Ma'lumotli/TOPIK/IELTS va karta o'sha darajaning
  Excel'iga qaraydi.
- Umumiy tugmadan yuklashda universitet katalogdagilar orasidan
  tanlanadi: univ_kod bir nechta universitetga mos kelsa (masalan,
  dhc - 대구보건대 va 동아보건대) jimgina birinchisiga yozilmaydi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVzniLdcRq9YV7e8nwFgs1
</commit_message>
<xml_diff>
--- a/public/templates/universitet-guideline-shablon.xlsx
+++ b/public/templates/universitet-guideline-shablon.xlsx
@@ -280,9 +280,9 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당.
+        <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당, kasbiy = kasbiy ta'lim (전문대학, 전문학사).
 Turi: tanlov
-Qiymatlar: bakalavr, transfer, magistratura, doktorantura, til_kursi
+Qiymatlar: bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy
 Namuna: bakalavr</t>
       </text>
     </comment>
@@ -1406,8 +1406,8 @@
     <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bahor, kuz" type="list">
       <formula1>"bahor,kuz"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bakalavr, transfer, magistratura, doktorantura, til_kursi" type="list">
-      <formula1>"bakalavr,transfer,magistratura,doktorantura,til_kursi"</formula1>
+    <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy" type="list">
+      <formula1>"bakalavr,transfer,magistratura,doktorantura,til_kursi,kasbiy"</formula1>
     </dataValidation>
     <dataValidation sqref="N2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: KRW, USD" type="list">
       <formula1>"KRW,USD"</formula1>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>bakalavr, transfer, magistratura, doktorantura, til_kursi</t>
+          <t>bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy</t>
         </is>
       </c>
       <c r="E44" s="14" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
-          <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당.</t>
+          <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당, kasbiy = kasbiy ta'lim (전문대학, 전문학사).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(universitetlar): kasbiy ta'lim Excel'i va bakalavr / magistr / kasbiy ta'lim filtri (#379)
- Excel shablonida yangi daraja: kasbiy (전문대학, 전문학사). Katalog
  sarlavhasiga "Excel kasbiy" tugmasi, universitet paneliga
  "Kasbiy ta'lim" yorlig'i qo'shildi. university_guidelines.daraja
  cheklovi kengaytirildi (migratsiya).
- Daraja filtri: Barcha darajalar / Bakalavr / Magistr / Kasbiy ta'lim,
  yonida natija soni bilan. Universitet qaysi darajada o'qitishi
  yuklangan Excel'dan va oliygoh turidan aniqlanadi: kollej - kasbiy
  ta'lim, 대학원대학교 - faqat magistr, qolganlari - bakalavr va magistr.
  Daraja tanlansa, Ma'lumotli/TOPIK/IELTS va karta o'sha darajaning
  Excel'iga qaraydi.
- Umumiy tugmadan yuklashda universitet katalogdagilar orasidan
  tanlanadi: univ_kod bir nechta universitetga mos kelsa (masalan,
  dhc - 대구보건대 va 동아보건대) jimgina birinchisiga yozilmaydi.


Claude-Session: https://claude.ai/code/session_01RVzniLdcRq9YV7e8nwFgs1

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/universitet-guideline-shablon.xlsx
+++ b/public/templates/universitet-guideline-shablon.xlsx
@@ -280,9 +280,9 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당.
+        <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당, kasbiy = kasbiy ta'lim (전문대학, 전문학사).
 Turi: tanlov
-Qiymatlar: bakalavr, transfer, magistratura, doktorantura, til_kursi
+Qiymatlar: bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy
 Namuna: bakalavr</t>
       </text>
     </comment>
@@ -1406,8 +1406,8 @@
     <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bahor, kuz" type="list">
       <formula1>"bahor,kuz"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bakalavr, transfer, magistratura, doktorantura, til_kursi" type="list">
-      <formula1>"bakalavr,transfer,magistratura,doktorantura,til_kursi"</formula1>
+    <dataValidation sqref="I2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy" type="list">
+      <formula1>"bakalavr,transfer,magistratura,doktorantura,til_kursi,kasbiy"</formula1>
     </dataValidation>
     <dataValidation sqref="N2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Noto'g'ri qiymat" error="Faqat: KRW, USD" type="list">
       <formula1>"KRW,USD"</formula1>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>bakalavr, transfer, magistratura, doktorantura, til_kursi</t>
+          <t>bakalavr, transfer, magistratura, doktorantura, til_kursi, kasbiy</t>
         </is>
       </c>
       <c r="E44" s="14" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
-          <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당.</t>
+          <t>Qabul darajasi. transfer = 편입학, til_kursi = 어학당, kasbiy = kasbiy ta'lim (전문대학, 전문학사).</t>
         </is>
       </c>
     </row>

</xml_diff>